<commit_message>
Audit /// Update V7
</commit_message>
<xml_diff>
--- a/app/gpl_audit/GPL.xlsx
+++ b/app/gpl_audit/GPL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/aj_mac/Documents/Atel/server/code/app/gpl_audit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D11152B-4D91-2E4B-BBDA-EA65C391E6FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18D9F6B3-FDC1-6F49-851C-66F4C357A1B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14380" yWindow="640" windowWidth="14420" windowHeight="16120" firstSheet="1" activeTab="5" xr2:uid="{0D659C63-0EA7-475F-99B7-E7E648DB9099}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="16080" firstSheet="1" activeTab="2" xr2:uid="{0D659C63-0EA7-475F-99B7-E7E648DB9099}"/>
   </bookViews>
   <sheets>
     <sheet name="TermPointToAmf" sheetId="2" r:id="rId1"/>
@@ -5741,7 +5741,7 @@
         <v>25</v>
       </c>
       <c r="O10" s="4" t="s">
-        <v>138</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -19699,7 +19699,7 @@
         <v>115</v>
       </c>
       <c r="F487" s="3">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G487" s="3" t="s">
         <v>578</v>

</xml_diff>